<commit_message>
Add/Update Quantities.xlsx via API
</commit_message>
<xml_diff>
--- a/BinancePTF/Quantities.xlsx
+++ b/BinancePTF/Quantities.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q734"/>
+  <dimension ref="A1:Q736"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29339,6 +29339,92 @@
       <c r="P734" t="inlineStr"/>
       <c r="Q734" t="inlineStr"/>
     </row>
+    <row r="735">
+      <c r="A735" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B735" t="n">
+        <v>0.00045565</v>
+      </c>
+      <c r="C735" t="n">
+        <v>1.21e-05</v>
+      </c>
+      <c r="D735" t="n">
+        <v>7.45e-06</v>
+      </c>
+      <c r="E735" t="n">
+        <v>3.635e-05</v>
+      </c>
+      <c r="F735" t="n">
+        <v>0.0003977</v>
+      </c>
+      <c r="G735" t="n">
+        <v>1863.22125016</v>
+      </c>
+      <c r="H735" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="I735" t="n">
+        <v>0.0004431</v>
+      </c>
+      <c r="J735" t="n">
+        <v>4663.85449423</v>
+      </c>
+      <c r="K735" t="n">
+        <v>0.83831888</v>
+      </c>
+      <c r="L735" t="n">
+        <v>0.14694965</v>
+      </c>
+      <c r="M735" t="inlineStr"/>
+      <c r="N735" t="inlineStr"/>
+      <c r="O735" t="inlineStr"/>
+      <c r="P735" t="inlineStr"/>
+      <c r="Q735" t="inlineStr"/>
+    </row>
+    <row r="736">
+      <c r="A736" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B736" t="n">
+        <v>0.00045565</v>
+      </c>
+      <c r="C736" t="n">
+        <v>1.21e-05</v>
+      </c>
+      <c r="D736" t="n">
+        <v>7.45e-06</v>
+      </c>
+      <c r="E736" t="n">
+        <v>3.635e-05</v>
+      </c>
+      <c r="F736" t="n">
+        <v>0.0003977</v>
+      </c>
+      <c r="G736" t="n">
+        <v>1863.22125016</v>
+      </c>
+      <c r="H736" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="I736" t="n">
+        <v>0.0004431</v>
+      </c>
+      <c r="J736" t="n">
+        <v>4663.85449423</v>
+      </c>
+      <c r="K736" t="n">
+        <v>0.83831888</v>
+      </c>
+      <c r="L736" t="n">
+        <v>0.14694965</v>
+      </c>
+      <c r="M736" t="inlineStr"/>
+      <c r="N736" t="inlineStr"/>
+      <c r="O736" t="inlineStr"/>
+      <c r="P736" t="inlineStr"/>
+      <c r="Q736" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>